<commit_message>
İş Takip Güncellemesi - 02.03.2026 09:13:56
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -2881,7 +2881,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L65" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="66">
@@ -2919,7 +2919,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L66" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="67">
@@ -2995,7 +2995,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L68" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="69">
@@ -3878,7 +3878,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L91" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="92">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 2.03.2026 10:21:00
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1665,7 +1665,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L33" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="34">
@@ -1741,7 +1741,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L35" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="36">
@@ -2235,7 +2235,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L48" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="49">
@@ -2273,7 +2273,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L49" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="50">
@@ -2311,7 +2311,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L50" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="51">
@@ -2349,7 +2349,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L51" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="52">
@@ -2387,7 +2387,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L52" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="53">
@@ -2463,7 +2463,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L54" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="55">
@@ -2501,7 +2501,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L55" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="56">
@@ -2539,7 +2539,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L56" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="57">
@@ -2577,7 +2577,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L57" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="58">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 2.03.2026 10:26:17
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1013,7 +1013,7 @@
         <v/>
       </c>
       <c r="L16" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
       <c r="M16" t="str">
         <v>10.02.2026 Araziye 12.02 de gidilecek</v>
@@ -1437,7 +1437,7 @@
         <v/>
       </c>
       <c r="L27" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ARAZİ DEVAM EDİYOR</v>
       </c>
     </row>
     <row r="28">
@@ -1513,7 +1513,7 @@
         <v/>
       </c>
       <c r="L29" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ARAZİ DEVAM EDİYOR</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 2.03.2026 10:28:38
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -823,7 +823,7 @@
         <v/>
       </c>
       <c r="L11" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="12">
@@ -1627,7 +1627,7 @@
         <v/>
       </c>
       <c r="L32" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 03.03.2026 08:12:47
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -519,7 +519,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L3" t="str">
-        <v>DEĞERLENDİRMEDE</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="4">
@@ -1013,7 +1013,7 @@
         <v/>
       </c>
       <c r="L16" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M16" t="str">
         <v>10.02.2026 Araziye 12.02 de gidilecek</v>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 3.03.2026 13:59:13
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4319,19 +4319,20 @@
         <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
       <c r="M102" t="str" xml:space="preserve">
-        <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d_
-07.11.2025 ormanı bakıp teslim edecek_x000d_
-10.11.2025 kontrol edilip firmaya teslim edilecek_x000d_
-10.11.2025 Ormancı 11.11.2025 teslim edecek_x000d_
-13.11.2025 Ormancı 17.11.2025 teslim edecek_x000d_
-20.11.2025 orman mükerrerliği ile ilgili beyanname düzenlendi tescili bekleniyor_x000d_
-02.12.2025 Krokilerine başlanıldı_x000d_
-15.12.2025 Proje hazırlanıyor_x000d_
-22.12.2025 Proje hazırlanıyor _x000d_
-05.01.2026 KROKİLERE BAŞLANACAK_x000d_
-15.01.2026 Devam ediyor firma_x000d_
-31.01.2026 Personel kontrolünde 09-13.02 askı ilanı yapılacak_x000d_
-26.02.2026 BİLGİLENDİRME İLANI YAPILACAK</v>
+        <v xml:space="preserve">01.11.2025 firmaya teslim edilecek
+07.11.2025 ormanı bakıp teslim edecek
+10.11.2025 kontrol edilip firmaya teslim edilecek
+10.11.2025 Ormancı 11.11.2025 teslim edecek
+13.11.2025 Ormancı 17.11.2025 teslim edecek
+20.11.2025 orman mükerrerliği ile ilgili beyanname düzenlendi tescili bekleniyor
+02.12.2025 Krokilerine başlanıldı
+15.12.2025 Proje hazırlanıyor
+22.12.2025 Proje hazırlanıyor 
+05.01.2026 KROKİLERE BAŞLANACAK
+15.01.2026 Devam ediyor firma
+31.01.2026 Personel kontrolünde 09-13.02 askı ilanı yapılacak
+26.02.2026 BİLGİLENDİRME İLANI YAPILACAK
+09.03.2026 askı ilanı</v>
       </c>
     </row>
     <row r="103">
@@ -5049,19 +5050,20 @@
         <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
       <c r="M118" t="str" xml:space="preserve">
-        <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d_
-05.11.2025 kontroller devam ediyor_x000d_
-31.01.2026 firma kroki hazırlıyor_x000d_
-10.11.2025 Değerlendrime 13.11.2025 de bitecek_x000d_
-13.11.2025 Firmaya 17-21 haftası teslim edilecek_x000d_
-20.11.2025 firmaya 24.11.2025 de teslim edilecek_x000d_
-02.12.2025 bugün firmaya teslim edilecek_x000d_
-15.12.2025 Proje hazırlanıyor_x000d_
-22.12.2025 Proje 25.12.2025 biticek, krokiler 30.12.2025 verilecek_x000d_
-02.01.2026 Firma projeyi hazırlıyor _x000d_
-15.01.2026 kroki hazırlanıyor_x000d_
-11.02.2026 Kroki kontrolü yapılıyor. Tutanak basılacak 16-20.02 askı_x000d_
-KROKİ/TUTANAK KONTROLLERİ 23.02 TAMAMLANIP 25.02.2026 İLAN YAPILACAK</v>
+        <v xml:space="preserve">01.11.2025 firmaya teslim edilecek
+05.11.2025 kontroller devam ediyor
+31.01.2026 firma kroki hazırlıyor
+10.11.2025 Değerlendrime 13.11.2025 de bitecek
+13.11.2025 Firmaya 17-21 haftası teslim edilecek
+20.11.2025 firmaya 24.11.2025 de teslim edilecek
+02.12.2025 bugün firmaya teslim edilecek
+15.12.2025 Proje hazırlanıyor
+22.12.2025 Proje 25.12.2025 biticek, krokiler 30.12.2025 verilecek
+02.01.2026 Firma projeyi hazırlıyor 
+15.01.2026 kroki hazırlanıyor
+11.02.2026 Kroki kontrolü yapılıyor. Tutanak basılacak 16-20.02 askı
+KROKİ/TUTANAK KONTROLLERİ 23.02 TAMAMLANIP 25.02.2026 İLAN YAPILACAK
+09.03.2026 askı ilanı</v>
       </c>
     </row>
     <row r="119" xml:space="preserve">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 3.03.2026 14:04:37
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4490,17 +4490,17 @@
         <v>BİLGİLENDİRME İLANINDA</v>
       </c>
       <c r="M106" t="str" xml:space="preserve">
-        <v xml:space="preserve">03.11.2025 firmaya teslim edilecek_x000d_
-05.11.2025 kontroller devam ediyor 10.11.2025 bazı yerlerin arazi kontrolleri yapılacak_x000d_
-13.11.2025 arazi kontrolü 18.11.2025 de yapılıp, 21.11.2025 de firmaya teslim edilecek_x000d_
-20.11.2025 arazi kontrolü yapılıyor 24.11.2025 de firmaya teslim edilecek_x000d_
-02.12.2025 krokileri hazırlanıyor_x000d_
-15.12.2025 Krokileri basılıyor_x000d_
-22.12.2025 Kroki kontrolü 25.12.2025 biticek_x000d_
-02.01.2026 Tutanaklarına başlanıldı_x000d_
-15.01.2026 TEMUR beyin kontrolünde_x000d_
-31.01.2026 03.02 askı yapılacak_x000d_
-BİLGİLENDİRME İLANINDA. KOMİSYON 26-27.02 YAPILIP KESİN ASKIYA 04.03 ÇIKILACAK</v>
+        <v xml:space="preserve">03.11.2025 firmaya teslim edilecek
+05.11.2025 kontroller devam ediyor 10.11.2025 bazı yerlerin arazi kontrolleri yapılacak
+13.11.2025 arazi kontrolü 18.11.2025 de yapılıp, 21.11.2025 de firmaya teslim edilecek
+20.11.2025 arazi kontrolü yapılıyor 24.11.2025 de firmaya teslim edilecek
+02.12.2025 krokileri hazırlanıyor
+15.12.2025 Krokileri basılıyor
+22.12.2025 Kroki kontrolü 25.12.2025 biticek
+02.01.2026 Tutanaklarına başlanıldı
+15.01.2026 TEMUR beyin kontrolünde
+31.01.2026 03.02 askı yapılacak
+BİLGİLENDİRME İLANINDA. KOMİSYON 26-27.02 YAPILIP KESİN ASKIYA 12.03 ÇIKILACAK</v>
       </c>
     </row>
     <row r="107" xml:space="preserve">
@@ -4715,16 +4715,16 @@
         <v>BİLGİLENDİRME İLANINDA</v>
       </c>
       <c r="M111" t="str" xml:space="preserve">
-        <v xml:space="preserve">24.10.2025 firmaya teslim edilecek_x000d_
-28.10.2025 firmaya teslim edilecek_x000d_
-03.11.2025 ormancı kontrolünde_x000d_
-20.11.2025 ormancı kontrolünde_x000d_
-02.12.2025 Firmaya teslim edildi_x000d_
-15.12.2025 Proje hazırlanıyor_x000d_
-22.12.2025 Kroki hazırlanıyor. 26.12.205 de biticek_x000d_
-02.01.2026 Kroki kontrolüne 05.01.2026 başlanıp 08.01.2026 bitip tutanağa geçilecek _x000d_
-15.01.2026 Tutanak başlanılacak_x000d_
-31.01.2026 imza aşamasında haftaiçi askı yapılacak_x000d_
+        <v xml:space="preserve">24.10.2025 firmaya teslim edilecek
+28.10.2025 firmaya teslim edilecek
+03.11.2025 ormancı kontrolünde
+20.11.2025 ormancı kontrolünde
+02.12.2025 Firmaya teslim edildi
+15.12.2025 Proje hazırlanıyor
+22.12.2025 Kroki hazırlanıyor. 26.12.205 de biticek
+02.01.2026 Kroki kontrolüne 05.01.2026 başlanıp 08.01.2026 bitip tutanağa geçilecek 
+15.01.2026 Tutanak başlanılacak
+31.01.2026 imza aşamasında haftaiçi askı yapılacak
 BİLGİLENDİRME İLANINDA. KOMİSYON 03-04.03 YAPILIP KESİN ASKIYA 09.03 ÇIKILACAK</v>
       </c>
     </row>
@@ -4853,14 +4853,14 @@
         <v>BİLGİLENDİRME İLANINDA</v>
       </c>
       <c r="M114" t="str" xml:space="preserve">
-        <v xml:space="preserve">14.11.2025 firmaya teslim edilecek_x000d_
-02.12.2025 araziye çıkılacak_x000d_
-15.12.2025 Kısmi arazi kontrolü yapılıp firmaya teslim edilecek(22.12.2025)_x000d_
-02.01.2026 Firmaya 05.01.2026 teslim edilecek_x000d_
-15.01.2026 Kroki kontrolünde_x000d_
-31.01.2026 Kroki müh. kontrolünde_x000d_
-11.02.2026 Askı imzalanıyor cuma asılacak_x000d_
-BİLGİLENDİRME İLANINDA. KOMİSYON 05-06.03 YAPILIP KESİN ASKIYA 11.03 ÇIKILACAK</v>
+        <v xml:space="preserve">14.11.2025 firmaya teslim edilecek
+02.12.2025 araziye çıkılacak
+15.12.2025 Kısmi arazi kontrolü yapılıp firmaya teslim edilecek(22.12.2025)
+02.01.2026 Firmaya 05.01.2026 teslim edilecek
+15.01.2026 Kroki kontrolünde
+31.01.2026 Kroki müh. kontrolünde
+11.02.2026 Askı imzalanıyor cuma asılacak
+BİLGİLENDİRME İLANINDA. KOMİSYON 05-06.03 YAPILIP KESİN ASKIYA 12.03 ÇIKILACAK</v>
       </c>
     </row>
     <row r="115" xml:space="preserve">
@@ -4901,14 +4901,15 @@
         <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
       <c r="M115" t="str" xml:space="preserve">
-        <v xml:space="preserve">Kıymetlendirmede eksiklikler var firma tamamlayacak bu hafta(20.10.2025)_x000d_
-05.11.2025 eksik uçuşlar teslim edildi_x000d_
-10.11.2025 kıymetlendirmeler kontrol ediliyor_x000d_
-13.11.2025 Firmaya 28.11.2025 de teslim edilecek_x000d_
-15.12.2025 Değerlendirme devam ediyor_x000d_
-22.12.2025 Kısmi uçuş yapıldı kıymetlendirme yapılıyor aynı zamanda değerlendirme devam ediyor_x000d_
-02.01.2026 Değerlendirme 15.01.2026 biticek_x000d_
-31.01.2026 firma projeyi hazırlıyor 16.02.2026 tamamlayacak_x000d_
+        <v xml:space="preserve">Kıymetlendirmede eksiklikler var firma tamamlayacak bu hafta(20.10.2025)
+05.11.2025 eksik uçuşlar teslim edildi
+10.11.2025 kıymetlendirmeler kontrol ediliyor
+13.11.2025 Firmaya 28.11.2025 de teslim edilecek
+15.12.2025 Değerlendirme devam ediyor
+22.12.2025 Kısmi uçuş yapıldı kıymetlendirme yapılıyor aynı zamanda değerlendirme devam ediyor
+02.01.2026 Değerlendirme 15.01.2026 biticek
+31.01.2026 firma projeyi hazırlıyor 16.02.2026 tamamlayacak
+12.03 askı
 KROKİ/TUTANAK KONTROLLERİ TAMAMLANIP 03.03.2026 İLAN YAPILACAK</v>
       </c>
     </row>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 05.03.2026 10:10:07
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1437,7 +1437,7 @@
         <v/>
       </c>
       <c r="L27" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="28">
@@ -1513,7 +1513,7 @@
         <v/>
       </c>
       <c r="L29" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 05.03.2026 13:06:34
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -5240,7 +5240,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L122" t="str">
-        <v>KOMİSYON AŞAMASINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M122" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 Tutanaklara başlanılacak_x000d_
@@ -9831,10 +9831,10 @@
         <v>2025-11-27</v>
       </c>
       <c r="N29" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O29" t="str">
-        <v/>
+        <v>2026-03-06</v>
       </c>
     </row>
     <row r="30">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 09.03.2026 00:02:43
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4375,7 +4375,7 @@
     </row>
     <row r="104">
       <c r="A104" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B104" t="str">
         <v>Toroslar</v>
@@ -4408,7 +4408,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L104" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
     </row>
     <row r="105">
@@ -4730,7 +4730,7 @@
     </row>
     <row r="112">
       <c r="A112" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B112" t="str">
         <v>Tarsus</v>
@@ -4763,7 +4763,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L112" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M112" t="str">
         <v>[x] 20.10.2025 askıya çıkacak</v>
@@ -4771,7 +4771,7 @@
     </row>
     <row r="113" xml:space="preserve">
       <c r="A113" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B113" t="str">
         <v>Tarsus</v>
@@ -4804,7 +4804,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L113" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M113" t="str" xml:space="preserve">
         <v xml:space="preserve">22.10.2025 firmaya teslim edilecek_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 09.03.2026 09:57:56
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4712,7 +4712,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L111" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M111" t="str" xml:space="preserve">
         <v xml:space="preserve">24.10.2025 firmaya teslim edilecek
@@ -9314,10 +9314,10 @@
         <v>2026-02-12</v>
       </c>
       <c r="N18" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O18" t="str">
-        <v/>
+        <v>2026-03-10</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 09.03.2026 09:59:57
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -2843,7 +2843,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L64" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="65">
@@ -2957,7 +2957,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L67" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="68">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 09.03.2026 11:16:26
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -481,7 +481,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L2" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="3">
@@ -557,7 +557,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L4" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="5">
@@ -671,7 +671,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L7" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 09.03.2026 11:45:32
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1209,7 +1209,7 @@
         <v/>
       </c>
       <c r="L21" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ARAZİ DEVAM EDİYOR</v>
       </c>
     </row>
     <row r="22">
@@ -1247,7 +1247,7 @@
         <v/>
       </c>
       <c r="L22" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 09.03.2026 13:06:10
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1931,7 +1931,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L40" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="41">
@@ -2425,7 +2425,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L53" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="54">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 10.03.2026 12:21:54
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -5048,7 +5048,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L118" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>BİLGİLENDİRME İLANINDA</v>
       </c>
       <c r="M118" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek
@@ -9634,13 +9634,13 @@
         <v>Yapıldı</v>
       </c>
       <c r="K25" t="str">
-        <v>Firmaya Teslim Edildi</v>
+        <v>Yapıldı</v>
       </c>
       <c r="L25" t="str">
         <v/>
       </c>
       <c r="M25" t="str">
-        <v/>
+        <v>2026-03-11</v>
       </c>
       <c r="N25" t="str">
         <v/>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 11.03.2026 12:06:20
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4316,7 +4316,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L102" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>BİLGİLENDİRME İLANINDA</v>
       </c>
       <c r="M102" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek
@@ -8882,13 +8882,13 @@
         <v>Yapıldı</v>
       </c>
       <c r="K9" t="str">
-        <v>Firmaya Teslim Edildi</v>
+        <v>Yapıldı</v>
       </c>
       <c r="L9" t="str">
         <v/>
       </c>
       <c r="M9" t="str">
-        <v/>
+        <v>2026-03-12</v>
       </c>
       <c r="N9" t="str">
         <v/>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 12.03.2026 08:43:48
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -3840,7 +3840,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L90" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="91">
@@ -3878,7 +3878,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L91" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="92">
@@ -3916,7 +3916,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L92" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="93">
@@ -3954,7 +3954,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L93" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="94">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 12.03.2026 08:45:17
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4487,7 +4487,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L106" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M106" t="str" xml:space="preserve">
         <v xml:space="preserve">03.11.2025 firmaya teslim edilecek_x000d_
@@ -9070,7 +9070,7 @@
         <v>Yapıldı</v>
       </c>
       <c r="K13" t="str">
-        <v>Firmaya Teslim Edildi</v>
+        <v>Yapıldı</v>
       </c>
       <c r="L13" t="str">
         <v/>
@@ -9079,10 +9079,10 @@
         <v>2026-02-04</v>
       </c>
       <c r="N13" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O13" t="str">
-        <v/>
+        <v>2026-03-13</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 12.03.2026 08:59:57
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4850,7 +4850,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L114" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M114" t="str" xml:space="preserve">
         <v xml:space="preserve">14.11.2025 firmaya teslim edilecek_x000d_
@@ -9455,10 +9455,10 @@
         <v>2026-02-17</v>
       </c>
       <c r="N21" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O21" t="str">
-        <v/>
+        <v>2026-03-13</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 17.03.2026 17:55:16
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4997,7 +4997,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L117" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M117" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -9596,10 +9596,10 @@
         <v>2026-02-24</v>
       </c>
       <c r="N24" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O24" t="str">
-        <v/>
+        <v>2026-03-18</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 26.03.2026 13:05:35
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1437,7 +1437,7 @@
         <v/>
       </c>
       <c r="L27" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="28">
@@ -1627,7 +1627,7 @@
         <v/>
       </c>
       <c r="L32" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 26.03.2026 13:37:51
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1703,7 +1703,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L34" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="35">
@@ -1779,7 +1779,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L36" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="37">
@@ -1817,7 +1817,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L37" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="38">
@@ -1855,7 +1855,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L38" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="39">
@@ -1969,7 +1969,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L41" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="42">
@@ -2045,7 +2045,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L43" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="44">
@@ -2083,7 +2083,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L44" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="45">
@@ -2159,7 +2159,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L46" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="47">
@@ -2235,7 +2235,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L48" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="49">
@@ -2273,7 +2273,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L49" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="50">
@@ -2311,7 +2311,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L50" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="51">
@@ -2501,7 +2501,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L55" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="56">
@@ -2577,7 +2577,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L57" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="58">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 02.04.2026 12:23:57
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -2653,7 +2653,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L59" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="60">
@@ -2691,7 +2691,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L60" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="61">
@@ -2767,7 +2767,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L62" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="63">
@@ -2919,7 +2919,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L66" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="67">
@@ -2957,7 +2957,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L67" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="68">
@@ -2995,7 +2995,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L68" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="69">
@@ -3267,7 +3267,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L75" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="76">
@@ -3305,7 +3305,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L76" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="77">
@@ -3343,7 +3343,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L77" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="78">
@@ -3381,7 +3381,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L78" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="79">
@@ -3419,7 +3419,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L79" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="80">
@@ -3457,7 +3457,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L80" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="81">
@@ -3536,7 +3536,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L82" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="83">
@@ -3574,7 +3574,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L83" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="84">
@@ -3612,7 +3612,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L84" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="85">
@@ -3688,7 +3688,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L86" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="87">
@@ -3726,7 +3726,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L87" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="88">
@@ -3764,7 +3764,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L88" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="89">
@@ -3802,7 +3802,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L89" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="90">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 02.04.2026 13:08:30
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -3153,7 +3153,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L72" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="73">
@@ -3650,7 +3650,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L85" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="86">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 6.04.2026 15:37:54
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4147,10 +4147,11 @@
         <v>FİRMAYA TESLİM EDİLDİ</v>
       </c>
       <c r="M98" t="str" xml:space="preserve">
-        <v xml:space="preserve">Ormancı kontrolünde(13.10.2025)_x000d__x000d_
-GM OLUR'u beklenecek_x000d__x000d_
-31.01.2026 kroki basılıyor_x000d__x000d_
-KROKİ/TUTANAK KONTROLLERİ TAMAMLANIP 02.03.2026 İLAN YAPILACAK</v>
+        <v xml:space="preserve">Ormancı kontrolünde(13.10.2025)
+GM OLUR'u beklenecek
+31.01.2026 kroki basılıyor
+KROKİ/TUTANAK KONTROLLERİ TAMAMLANIP 02.03.2026 İLAN YAPILACAK
+Eksik krokiler tamamlanıyor. Geçici-8 kullanıcı yazılmayan var. 06.04.2026</v>
       </c>
     </row>
     <row r="99">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 13.04.2026 14:07:22
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4230,7 +4230,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L100" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M100" t="str" xml:space="preserve">
         <v xml:space="preserve">15.10.2025 Projesine başlanılacak(Ormancı kontrolünde)_x000d__x000d_
@@ -8801,10 +8801,10 @@
         <v>2026-01-30</v>
       </c>
       <c r="N7" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O7" t="str">
-        <v/>
+        <v>2026-04-14</v>
       </c>
     </row>
     <row r="8">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 14.04.2026 10:21:46
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1054,7 +1054,7 @@
         <v/>
       </c>
       <c r="L17" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
       <c r="M17" t="str">
         <v>10.02.2026 Araziye 11.02 de gidilecek</v>
@@ -1209,7 +1209,7 @@
         <v/>
       </c>
       <c r="L21" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>DEĞERLENDİRMEDE</v>
       </c>
     </row>
     <row r="22">
@@ -1551,7 +1551,7 @@
         <v/>
       </c>
       <c r="L30" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ARAZİ DEVAM EDİYOR</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 14.04.2026 10:24:50
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1285,7 +1285,7 @@
         <v/>
       </c>
       <c r="L23" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="24">
@@ -1589,7 +1589,7 @@
         <v/>
       </c>
       <c r="L31" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>İHALEDEN/PROGRAMDAN ÇIKARILDI</v>
       </c>
       <c r="M31" t="str">
         <v>Mahkeme ile orman olmuş çıkarılacak</v>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 21.04.2026 23:51:08
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4952,7 +4952,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L116" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>BİLGİLENDİRME İLANINDA</v>
       </c>
       <c r="M116" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -9544,13 +9544,13 @@
         <v>Yapıldı</v>
       </c>
       <c r="K23" t="str">
-        <v>Devam Ediyor</v>
+        <v>Yapıldı</v>
       </c>
       <c r="L23" t="str">
         <v/>
       </c>
       <c r="M23" t="str">
-        <v/>
+        <v>2026-04-22</v>
       </c>
       <c r="N23" t="str">
         <v/>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 21.04.2026 23:53:48
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4320,7 +4320,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L102" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KOMİSYON AŞAMASINDA</v>
       </c>
       <c r="M102" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d_
@@ -4458,7 +4458,7 @@
     </row>
     <row r="106" xml:space="preserve">
       <c r="A106" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B106" t="str">
         <v>Tarsus</v>
@@ -4491,7 +4491,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L106" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M106" t="str" xml:space="preserve">
         <v xml:space="preserve">03.11.2025 firmaya teslim edilecek_x000d_
@@ -4509,7 +4509,7 @@
     </row>
     <row r="107" xml:space="preserve">
       <c r="A107" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B107" t="str">
         <v>Tarsus</v>
@@ -4542,7 +4542,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L107" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M107" t="str" xml:space="preserve">
         <v xml:space="preserve">16.10.2025 firmaya teslim edilecek_x000d__x000d_
@@ -4635,7 +4635,7 @@
     </row>
     <row r="110" xml:space="preserve">
       <c r="A110" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B110" t="str">
         <v>Tarsus</v>
@@ -4668,7 +4668,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L110" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M110" t="str" xml:space="preserve">
         <v xml:space="preserve">16.10.2025 Taşçılı tutanak Kadastro Üyesine teslim edilecek._x000d__x000d_
@@ -4683,7 +4683,7 @@
     </row>
     <row r="111" xml:space="preserve">
       <c r="A111" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B111" t="str">
         <v>Tarsus</v>
@@ -4716,7 +4716,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L111" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M111" t="str" xml:space="preserve">
         <v xml:space="preserve">24.10.2025 firmaya teslim edilecek_x000d_
@@ -4821,7 +4821,7 @@
     </row>
     <row r="114" xml:space="preserve">
       <c r="A114" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B114" t="str">
         <v>Tarsus</v>
@@ -4854,7 +4854,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L114" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M114" t="str" xml:space="preserve">
         <v xml:space="preserve">14.11.2025 firmaya teslim edilecek_x000d_
@@ -4968,7 +4968,7 @@
     </row>
     <row r="117" xml:space="preserve">
       <c r="A117" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B117" t="str">
         <v>Toroslar</v>
@@ -5001,7 +5001,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L117" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M117" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -5052,7 +5052,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L118" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KOMİSYON AŞAMASINDA</v>
       </c>
       <c r="M118" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d_
@@ -5106,7 +5106,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L119" t="str">
-        <v>FİRMAYA TESLİM EDİLDİ</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
       <c r="M119" t="str" xml:space="preserve">
         <v xml:space="preserve">15.12.2025 Değerlendirme devam ediyor_x000d__x000d_
@@ -5195,7 +5195,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L121" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KOMİSYON AŞAMASINDA</v>
       </c>
       <c r="M121" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 firmaya teslim edilecek_x000d__x000d_
@@ -5211,7 +5211,7 @@
     </row>
     <row r="122" xml:space="preserve">
       <c r="A122" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B122" t="str">
         <v>Yenişehir</v>
@@ -5244,7 +5244,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L122" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M122" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 Tutanaklara başlanılacak_x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 27.04.2026 16:20:30
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1054,7 +1054,7 @@
         <v/>
       </c>
       <c r="L17" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M17" t="str">
         <v>10.02.2026 Araziye 11.02 de gidilecek</v>
@@ -1095,7 +1095,7 @@
         <v/>
       </c>
       <c r="L18" t="str">
-        <v>DEĞERLENDİRMEDE</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="19">
@@ -1133,7 +1133,7 @@
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>ARAZİ DEVAM EDİYOR</v>
       </c>
     </row>
     <row r="20">
@@ -1361,7 +1361,7 @@
         <v/>
       </c>
       <c r="L25" t="str">
-        <v>DEĞERLENDİRMEDE</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 29.04.2026 13:30:31
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -5195,7 +5195,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L121" t="str">
-        <v>KOMİSYON AŞAMASINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M121" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 firmaya teslim edilecek_x000d__x000d_
@@ -9788,10 +9788,10 @@
         <v>2025-12-09</v>
       </c>
       <c r="N28" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O28" t="str">
-        <v/>
+        <v>2026-04-30</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 29.04.2026 15:03:49
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -5052,7 +5052,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L118" t="str">
-        <v>KOMİSYON AŞAMASINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M118" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d_
@@ -9647,10 +9647,10 @@
         <v>2026-03-11</v>
       </c>
       <c r="N25" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O25" t="str">
-        <v/>
+        <v>2026-04-30</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 30.04.2026 12:43:26
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -481,7 +481,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L2" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="3">
@@ -557,7 +557,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L4" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="5">
@@ -595,7 +595,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L5" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="6">
@@ -633,7 +633,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L6" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="7">
@@ -671,7 +671,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L7" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="8">
@@ -709,7 +709,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L8" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="9">
@@ -747,7 +747,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L9" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="10">
@@ -785,7 +785,7 @@
         <v>2025-10-29</v>
       </c>
       <c r="L10" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="11">
@@ -1668,7 +1668,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L33" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="34">
@@ -1744,7 +1744,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L35" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="36">
@@ -1896,7 +1896,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L39" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="40">
@@ -1934,7 +1934,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L40" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="41">
@@ -2010,7 +2010,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L42" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="43">
@@ -2124,7 +2124,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L45" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="46">
@@ -2200,7 +2200,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L47" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="48">
@@ -2352,7 +2352,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L51" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="52">
@@ -2390,7 +2390,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L52" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="53">
@@ -2428,7 +2428,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L53" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="54">
@@ -2466,7 +2466,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L54" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="55">
@@ -2542,7 +2542,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L56" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="57">
@@ -2618,7 +2618,7 @@
         <v>2025-10-31</v>
       </c>
       <c r="L58" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="59">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 08.05.2026 10:01:30
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -899,7 +899,7 @@
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>DEĞERLENDİRMEDE</v>
       </c>
     </row>
     <row r="14">
@@ -1095,7 +1095,7 @@
         <v/>
       </c>
       <c r="L18" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="19">
@@ -1133,7 +1133,7 @@
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>DEĞERLENDİRMEDE</v>
       </c>
     </row>
     <row r="20">
@@ -1209,7 +1209,7 @@
         <v/>
       </c>
       <c r="L21" t="str">
-        <v>DEĞERLENDİRMEDE</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="22">
@@ -1285,7 +1285,7 @@
         <v/>
       </c>
       <c r="L23" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 08.05.2026 12:20:12
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -7879,7 +7879,7 @@
     </row>
     <row r="192">
       <c r="A192" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B192" t="str">
         <v>Silifke</v>
@@ -7912,7 +7912,7 @@
         <v/>
       </c>
       <c r="L192" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="193">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 18.05.2026 14:37:56
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -9553,10 +9553,10 @@
         <v>2026-04-22</v>
       </c>
       <c r="N23" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O23" t="str">
-        <v/>
+        <v>2026-05-20</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 20.05.2026 12:40:02
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4320,7 +4320,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L102" t="str">
-        <v>KOMİSYON AŞAMASINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M102" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d_
@@ -4952,7 +4952,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L116" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M116" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -8895,10 +8895,10 @@
         <v>2026-03-12</v>
       </c>
       <c r="N9" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O9" t="str">
-        <v/>
+        <v>2026-05-21</v>
       </c>
     </row>
     <row r="10">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 20.05.2026 12:41:32
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4197,7 +4197,7 @@
     </row>
     <row r="100" xml:space="preserve">
       <c r="A100" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B100" t="str">
         <v>Toroslar</v>
@@ -4230,7 +4230,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L100" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M100" t="str" xml:space="preserve">
         <v xml:space="preserve">15.10.2025 Projesine başlanılacak(Ormancı kontrolünde)_x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 22.05.2026 08:42:54
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -823,7 +823,7 @@
         <v/>
       </c>
       <c r="L11" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="12">
@@ -861,7 +861,7 @@
         <v/>
       </c>
       <c r="L12" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="13">
@@ -1013,7 +1013,7 @@
         <v/>
       </c>
       <c r="L16" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M16" t="str">
         <v>10.02.2026 Araziye 12.02 de gidilecek</v>
@@ -1399,7 +1399,7 @@
         <v/>
       </c>
       <c r="L26" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="27">
@@ -1475,7 +1475,7 @@
         <v/>
       </c>
       <c r="L28" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 22.05.2026 09:23:27
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -899,7 +899,7 @@
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>DEĞERLENDİRMEDE</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="14">
@@ -937,7 +937,7 @@
         <v/>
       </c>
       <c r="L14" t="str">
-        <v>DEĞERLENDİRMEDE</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="15">
@@ -1171,7 +1171,7 @@
         <v/>
       </c>
       <c r="L20" t="str">
-        <v>ÇALIŞMA ALANI İLANI YAPILDI</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="21">
@@ -1323,7 +1323,7 @@
         <v/>
       </c>
       <c r="L24" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 31.05.2026 14:40:09
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4071,7 +4071,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L96" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="97">
@@ -4279,7 +4279,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L101" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M101" t="str">
         <v/>
@@ -4374,7 +4374,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L103" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="104">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 02.06.2026 09:27:52
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1437,7 +1437,7 @@
         <v/>
       </c>
       <c r="L27" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="28">
@@ -1513,7 +1513,7 @@
         <v/>
       </c>
       <c r="L29" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="30">
@@ -1630,7 +1630,7 @@
         <v/>
       </c>
       <c r="L32" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 02.06.2026 15:56:23
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4902,7 +4902,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L115" t="str">
-        <v>KOMİSYON AŞAMASINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M115" t="str" xml:space="preserve">
         <v xml:space="preserve">Kıymetlendirmede eksiklikler var firma tamamlayacak bu hafta(20.10.2025)_x000d_
@@ -9506,10 +9506,10 @@
         <v>2026-03-17</v>
       </c>
       <c r="N22" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O22" t="str">
-        <v/>
+        <v>2026-06-03</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 09.06.2026 10:41:49
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -899,7 +899,7 @@
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="14">
@@ -1171,7 +1171,7 @@
         <v/>
       </c>
       <c r="L20" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="21">
@@ -1323,7 +1323,7 @@
         <v/>
       </c>
       <c r="L24" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 11.06.2026 10:38:57
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4279,7 +4279,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L101" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M101" t="str">
         <v/>
@@ -4374,7 +4374,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L103" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="104">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 11.06.2026 10:40:22
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -5052,7 +5052,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L118" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M118" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d_
@@ -5195,7 +5195,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L121" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M121" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 firmaya teslim edilecek_x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 12.06.2026 12:51:14
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4192,7 +4192,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L99" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="100" xml:space="preserve">
@@ -4412,7 +4412,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L104" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="105">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 12.06.2026 12:52:16
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -5019,7 +5019,7 @@
     </row>
     <row r="118" xml:space="preserve">
       <c r="A118" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B118" t="str">
         <v>Toroslar</v>
@@ -5162,7 +5162,7 @@
     </row>
     <row r="121" xml:space="preserve">
       <c r="A121" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B121" t="str">
         <v>Toroslar</v>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 16.06.2026 09:53:48
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -899,7 +899,7 @@
         <v/>
       </c>
       <c r="L13" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="14">
@@ -1323,7 +1323,7 @@
         <v/>
       </c>
       <c r="L24" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 16.06.2026 09:54:42
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -975,7 +975,7 @@
         <v/>
       </c>
       <c r="L15" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="16">
@@ -1133,7 +1133,7 @@
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>FİRMAYA TESLİM EDİLDİ</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="20">
@@ -1551,7 +1551,7 @@
         <v/>
       </c>
       <c r="L30" t="str">
-        <v>ARAZİ DEVAM EDİYOR</v>
+        <v>KROKİ/TUTANAK KONTROLÜ</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 19.06.2026 09:06:58
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1437,7 +1437,7 @@
         <v/>
       </c>
       <c r="L27" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="28">
@@ -1513,7 +1513,7 @@
         <v/>
       </c>
       <c r="L29" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="30">
@@ -1630,7 +1630,7 @@
         <v/>
       </c>
       <c r="L32" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="33">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 23.06.2026 09:35:24
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -1133,7 +1133,7 @@
         <v/>
       </c>
       <c r="L19" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="20">
@@ -1171,7 +1171,7 @@
         <v/>
       </c>
       <c r="L20" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 25.06.2026 08:08:26
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4147,7 +4147,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L98" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>BİLGİLENDİRME İLANINDA</v>
       </c>
       <c r="M98" t="str" xml:space="preserve">
         <v xml:space="preserve">Ormancı kontrolünde(13.10.2025)_x000d_
@@ -8736,13 +8736,13 @@
         <v>Yapıldı</v>
       </c>
       <c r="K5" t="str">
-        <v>Devam Ediyor</v>
+        <v>Yapıldı</v>
       </c>
       <c r="L5" t="str">
         <v/>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>2026-06-26</v>
       </c>
       <c r="N5" t="str">
         <v/>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 25.06.2026 08:08:51
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4287,7 +4287,7 @@
     </row>
     <row r="102" xml:space="preserve">
       <c r="A102" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B102" t="str">
         <v>Toroslar</v>
@@ -4320,7 +4320,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L102" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M102" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 25.06.2026 08:09:27
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4919,7 +4919,7 @@
     </row>
     <row r="116" xml:space="preserve">
       <c r="A116" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B116" t="str">
         <v>Mezitli</v>
@@ -4952,7 +4952,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L116" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M116" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 04.07.2026 17:31:48
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4869,7 +4869,7 @@
     </row>
     <row r="115" xml:space="preserve">
       <c r="A115" t="str">
-        <v>HAYIR</v>
+        <v>EVET</v>
       </c>
       <c r="B115" t="str">
         <v>Tarsus</v>
@@ -4902,7 +4902,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L115" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
       </c>
       <c r="M115" t="str" xml:space="preserve">
         <v xml:space="preserve">Kıymetlendirmede eksiklikler var firma tamamlayacak bu hafta(20.10.2025)_x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 05.07.2026 16:14:12
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4450,7 +4450,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L105" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M105" t="str">
         <v>[x] 21.10.2025 komisyon yapılacak(İsmail Pehlivan)</v>
@@ -4491,7 +4491,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L106" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M106" t="str" xml:space="preserve">
         <v xml:space="preserve">03.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -4542,7 +4542,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L107" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M107" t="str" xml:space="preserve">
         <v xml:space="preserve">16.10.2025 firmaya teslim edilecek_x000d__x000d__x000d_
@@ -4630,7 +4630,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L109" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
     </row>
     <row r="110" xml:space="preserve">
@@ -4668,7 +4668,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L110" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M110" t="str" xml:space="preserve">
         <v xml:space="preserve">16.10.2025 Taşçılı tutanak Kadastro Üyesine teslim edilecek._x000d__x000d__x000d_
@@ -4716,7 +4716,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L111" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M111" t="str" xml:space="preserve">
         <v xml:space="preserve">24.10.2025 firmaya teslim edilecek_x000d__x000d_
@@ -4808,7 +4808,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L113" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M113" t="str" xml:space="preserve">
         <v xml:space="preserve">22.10.2025 firmaya teslim edilecek_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 10.07.2026 11:47:33
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -937,7 +937,7 @@
         <v/>
       </c>
       <c r="L14" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="15">
@@ -975,7 +975,7 @@
         <v/>
       </c>
       <c r="L15" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="16">
@@ -1551,7 +1551,7 @@
         <v/>
       </c>
       <c r="L30" t="str">
-        <v>KROKİ/TUTANAK KONTROLÜ</v>
+        <v>ASKI İLANINA HAZIRLANIYOR</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 14.07.2026 08:13:52
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -975,7 +975,7 @@
         <v/>
       </c>
       <c r="L15" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="16">
@@ -1551,7 +1551,7 @@
         <v/>
       </c>
       <c r="L30" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>KESİN ASKIDA</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 20.07.2026 11:24:43
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4230,7 +4230,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L100" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M100" t="str" xml:space="preserve">
         <v xml:space="preserve">15.10.2025 Projesine başlanılacak(Ormancı kontrolünde)_x000d__x000d__x000d_
@@ -4767,7 +4767,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L112" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M112" t="str">
         <v>[x] 20.10.2025 askıya çıkacak</v>
@@ -4854,7 +4854,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L114" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M114" t="str" xml:space="preserve">
         <v xml:space="preserve">14.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -5052,7 +5052,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L118" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M118" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 21.07.2026 14:14:28
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4589,7 +4589,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L108" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M108" t="str">
         <v>[x] 21.10.2025 komisyon yapılacak(Lokman)</v>
@@ -4630,7 +4630,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L109" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="110" xml:space="preserve">
@@ -4808,7 +4808,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L113" t="str">
-        <v>DEVİR YAPILDI</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
       <c r="M113" t="str" xml:space="preserve">
         <v xml:space="preserve">22.10.2025 firmaya teslim edilecek_x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 29.07.2026 10:56:16
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -7801,7 +7801,7 @@
         <v/>
       </c>
       <c r="L189" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="190">
@@ -7839,7 +7839,7 @@
         <v/>
       </c>
       <c r="L190" t="str">
-        <v>KESİN ASKIDA</v>
+        <v>TESCİLİ BİTTİ</v>
       </c>
     </row>
     <row r="191">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 31.07.2026 17:18:21
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -5052,7 +5052,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L118" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M118" t="str" xml:space="preserve">
         <v xml:space="preserve">01.11.2025 firmaya teslim edilecek_x000d__x000d_
@@ -5195,7 +5195,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L121" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M121" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 firmaya teslim edilecek_x000d__x000d__x000d_

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 03.08.2026 11:03:53
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -5106,7 +5106,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L119" t="str">
-        <v>ASKI İLANINA HAZIRLANIYOR</v>
+        <v>BİLGİLENDİRME İLANINDA</v>
       </c>
       <c r="M119" t="str" xml:space="preserve">
         <v xml:space="preserve">15.12.2025 Değerlendirme devam ediyor_x000d__x000d__x000d_
@@ -9732,7 +9732,7 @@
         <v/>
       </c>
       <c r="M26" t="str">
-        <v/>
+        <v>2026-08-04</v>
       </c>
       <c r="N26" t="str">
         <v/>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 12.08.2026 09:21:16
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4147,7 +4147,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L98" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M98" t="str" xml:space="preserve">
         <v xml:space="preserve">Ormancı kontrolünde(13.10.2025)_x000d_
@@ -8748,10 +8748,10 @@
         <v>2026-06-26</v>
       </c>
       <c r="N5" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O5" t="str">
-        <v/>
+        <v>2026-08-12</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 27.08.2026 13:31:01
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -7555,7 +7555,7 @@
         <v>GÜNCELLEME</v>
       </c>
       <c r="E183" t="str">
-        <v>SARİYE KUŞÇU, ŞEHMUS ÖZTÜRK, MÜJDE TÜKMEN, ENDER NUSRET ÖNAL GÜLSOY, İSMAİL AKLAN</v>
+        <v>SARİYE KUŞÇU, ŞEHMUS ÖZTÜRK, MÜJDE TÜRKMEN, ENDER NUSRET ÖNAL GÜLSOY, İSMAİL AKLAN</v>
       </c>
       <c r="F183" t="str">
         <v>4</v>
@@ -7593,7 +7593,7 @@
         <v>GÜNCELLEME</v>
       </c>
       <c r="E184" t="str">
-        <v>SARİYE KUŞÇU, ŞEHMUS ÖZTÜRK, MÜJDE TÜKMEN, ENDER NUSRET ÖNAL GÜLSOY, İSMAİL AKLAN</v>
+        <v>SARİYE KUŞÇU, ŞEHMUS ÖZTÜRK, MÜJDE TÜRKMEN, ENDER NUSRET ÖNAL GÜLSOY, İSMAİL AKLAN</v>
       </c>
       <c r="F184" t="str">
         <v>1</v>

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 07.09.2026 15:42:08
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -9738,10 +9738,10 @@
         <v>2026-08-04</v>
       </c>
       <c r="N26" t="str">
-        <v/>
+        <v>Yapıldı</v>
       </c>
       <c r="O26" t="str">
-        <v/>
+        <v>2026-09-04</v>
       </c>
     </row>
     <row r="27">

</xml_diff>

<commit_message>
İş Takip Güncellemesi - 07.09.2026 16:29:04
</commit_message>
<xml_diff>
--- a/istakip.xlsx
+++ b/istakip.xlsx
@@ -4902,7 +4902,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L115" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M115" t="str" xml:space="preserve">
         <v xml:space="preserve">Kıymetlendirmede eksiklikler var firma tamamlayacak bu hafta(20.10.2025)_x000d__x000d_
@@ -5106,7 +5106,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L119" t="str">
-        <v>BİLGİLENDİRME İLANINDA</v>
+        <v>KESİN ASKIDA</v>
       </c>
       <c r="M119" t="str" xml:space="preserve">
         <v xml:space="preserve">15.12.2025 Değerlendirme devam ediyor_x000d__x000d__x000d_
@@ -5244,7 +5244,7 @@
         <v>2025-05-23</v>
       </c>
       <c r="L122" t="str">
-        <v>KESİN ASKIDAN İNDİ. BEKLEMEDE</v>
+        <v>DEVİR YAPILDI</v>
       </c>
       <c r="M122" t="str" xml:space="preserve">
         <v xml:space="preserve">17.10.2025 Tutanaklara başlanılacak_x000d__x000d__x000d_

</xml_diff>